<commit_message>
Add purchase-list attributes and investigation scenarios
The importer reads origin_country, customs_required and permit_required
on tasks and an optional Procurement sheet (item, supplier, origin,
quantity, incoterms, customs, certification, planned arrival, needed-for
task). The hero workbook gains those values; calculators do not read
them, so H04 and REPLAY are unchanged.

Adds the X2, X2-control, N-X2, X1-A and X1-B scenario data. External
notices load through the same path as a registered-source scan, marked
SYNTHETIC, so their automatic analysis stays rules-only. The API image
and compose now ship the scenario file and the replay cassette.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/l1_project/hero_battery_factory_project.xlsx
+++ b/data/l1_project/hero_battery_factory_project.xlsx
@@ -11,6 +11,7 @@
     <sheet name="WBS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Partners" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Risk Profile" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Procurement" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -597,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V65"/>
+  <dimension ref="A1:Y65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -735,6 +736,21 @@
           <t>data_origin</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>origin_country</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>customs_required</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>permit_required</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1939,6 +1955,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2039,6 +2060,11 @@
       <c r="V14" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>예</t>
         </is>
       </c>
     </row>
@@ -2245,6 +2271,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2347,6 +2378,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3689,6 +3725,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4407,6 +4448,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4509,6 +4555,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4615,6 +4666,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4717,6 +4773,11 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4819,6 +4880,16 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4921,6 +4992,16 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5023,6 +5104,16 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -5125,6 +5216,16 @@
           <t>SYNTHETIC</t>
         </is>
       </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6563,6 +6664,11 @@
       <c r="V58" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>예</t>
         </is>
       </c>
     </row>
@@ -7923,4 +8029,370 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>item_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>item_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>supplier_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>origin_country</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>incoterms</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>customs_required</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>permit_or_certification</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>planned_arrival</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>needed_for_task_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>P-A1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>[합성] 셀 설비 1차 선적(코팅·권취·조립기)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Equipment Vendor A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CE 적합성 선언, 원산지 증명</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>T044</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P-A2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[합성] 모듈·팩 설비</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Equipment Vendor B</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CE 적합성 선언</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>T044</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P-B</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[합성] 셀 설비 작업자 교육 키트(운전 시뮬레이터)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Equipment Vendor A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>CE 적합성 선언</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>T058</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P-C</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>[합성] 셀 라인 교정·계측 장비 세트</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Equipment Vendor A</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>교정 성적서, CE 적합성 선언</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>T051</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P-D</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>[합성] 모듈 라인 시운전 예비 부품</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Equipment Vendor B</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CE 적합성 선언</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2027-04-30</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>T054</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P-E</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>[합성] 변전 설비(변압기·개폐기)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Utility Provider</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DDP</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>계통 연계 승인</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>T029</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Base X1-A and X2 on real L2 cases and show the source
X1-A now follows RS-001 (installation and validation technicians leaving
after an immigration raid at the Hyundai-LG battery plant): work-permit
verification for non-EU installation and commissioning technicians,
affecting Vendor A's on-site tasks. X2 follows RS-019 (China's
per-shipment export licences for rare-earth magnets): the supplier's
magnet parts wait for a licence, and the later magnet-bearing items P-B
and P-C need licences of their own. Dates stay synthetic; article delay
lengths are not used as inputs.

The investigation result lists the real article (title, outlet,
publication date, link) outside the model's input, and a confirmation
question that omits the calculated deadline gets it appended.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/l1_project/hero_battery_factory_project.xlsx
+++ b/data/l1_project/hero_battery_factory_project.xlsx
@@ -8100,7 +8100,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[합성] 셀 설비 1차 선적(코팅·권취·조립기)</t>
+          <t>[합성] 셀 설비 1차 선적 서보 모터 자석 부품(중국 공장 직송)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CE 적합성 선언, 원산지 증명</t>
+          <t>중국 희토류 수출 허가(선적마다), 원산지 증명</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[합성] 셀 설비 작업자 교육 키트(운전 시뮬레이터)</t>
+          <t>[합성] 셀 설비 교육 시뮬레이터 구동부(서보 모터·희토류 자석 포함)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CE 적합성 선언</t>
+          <t>중국 희토류 수출 허가(선적마다)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[합성] 셀 라인 교정·계측 장비 세트</t>
+          <t>[합성] 셀 라인 교정용 정밀 서보 스테이지(희토류 자석 포함)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>교정 성적서, CE 적합성 선언</t>
+          <t>중국 희토류 수출 허가(선적마다), 교정 성적서</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">

</xml_diff>